<commit_message>
Landing anti-macet: keep-warm GAS, retry timeout abort, dedup wave + tab Sesi admin & lembar
</commit_message>
<xml_diff>
--- a/DATA TES BERSAMA_DATA SHEET INTERNAL KSP.xlsx
+++ b/DATA TES BERSAMA_DATA SHEET INTERNAL KSP.xlsx
@@ -15,6 +15,7 @@
     <sheet name="kedatangan" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="pengumuman" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="lembar" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sesi" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -777,6 +778,168 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>cabang_id</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>sesi</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>jenjang</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>waktu</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>tampil</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sesi 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>07.30–08.30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sesi 2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SMP &amp; SMA (Akhwat)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>09.15–10.15</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sesi 3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SMP &amp; SMA (Ikhwan)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>11.00–12.00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S1-AW3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AW3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sesi 1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>07.30–08.30</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1844,32 +2007,32 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>P105</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>Anas Ubaid</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>AW1</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>085921026401</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="0" t="inlineStr">
         <is>
           <t>M4</t>
         </is>
@@ -27414,46 +27577,46 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>P104</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>Dewi Lestari</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>penguji</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr"/>
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>P105</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>Anas Ubaid</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>penguji</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr"/>
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>P5</t>
         </is>

</xml_diff>